<commit_message>
berlin isn't running properly (getting infeasible solution in an unexpected way) so going to run with leaving berlin out for now and figure out berlin later. checked run for other cases
</commit_message>
<xml_diff>
--- a/workforce_size/schedule_thesis/method_region0_run.xlsx
+++ b/workforce_size/schedule_thesis/method_region0_run.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R3"/>
+  <dimension ref="A1:S2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -515,10 +515,15 @@
       </c>
       <c r="Q1" s="1" t="inlineStr">
         <is>
+          <t>obj_val_next</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
           <t>number_of_trials</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>log_ind</t>
         </is>
@@ -526,11 +531,11 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>20000</v>
+        <v>11252</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>lyon</t>
+          <t>frankfurt</t>
         </is>
       </c>
       <c r="C2" t="n">
@@ -538,113 +543,54 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>fixed</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr"/>
+          <t>partflex</t>
+        </is>
+      </c>
+      <c r="E2" t="n">
+        <v>3</v>
+      </c>
       <c r="F2" t="n">
-        <v>1.2</v>
+        <v>1.8</v>
       </c>
       <c r="G2" t="n">
-        <v>0.75</v>
+        <v>1.5</v>
       </c>
       <c r="H2" t="n">
-        <v>0.6</v>
+        <v>0.8</v>
       </c>
       <c r="I2" t="n">
         <v>0</v>
       </c>
       <c r="J2" t="n">
-        <v>219329</v>
+        <v>152795</v>
       </c>
       <c r="K2" t="inlineStr">
         <is>
+          <t>{'0': 0, '1': 2, '2': 4}</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
           <t>{'0': 0, '1': 4}</t>
         </is>
       </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>{'0': 0, '1': 4}</t>
-        </is>
-      </c>
       <c r="M2" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="N2" s="2" t="n">
-        <v>45593.71702709381</v>
-      </c>
-      <c r="O2" t="n">
-        <v>2850.593333333358</v>
-      </c>
+        <v>45599.66117506041</v>
+      </c>
+      <c r="O2" t="inlineStr"/>
       <c r="P2" t="n">
-        <v>2850.593333333357</v>
+        <v>2478.32000000007</v>
       </c>
       <c r="Q2" t="n">
-        <v>15</v>
+        <v>2480.14000000007</v>
       </c>
       <c r="R2" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="n">
-        <v>20020</v>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>lyon</t>
-        </is>
-      </c>
-      <c r="C3" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>fixed</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr"/>
-      <c r="F3" t="n">
-        <v>1.2</v>
-      </c>
-      <c r="G3" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="H3" t="n">
-        <v>0.7</v>
-      </c>
-      <c r="I3" t="n">
-        <v>0</v>
-      </c>
-      <c r="J3" t="n">
-        <v>219329</v>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>{'0': 0, '1': 4}</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>{'0': 0, '1': 4}</t>
-        </is>
-      </c>
-      <c r="M3" t="n">
-        <v>15</v>
-      </c>
-      <c r="N3" s="2" t="n">
-        <v>45593.7172760728</v>
-      </c>
-      <c r="O3" t="n">
-        <v>2850.593333333358</v>
-      </c>
-      <c r="P3" t="n">
-        <v>2850.593333333357</v>
-      </c>
-      <c r="Q3" t="n">
-        <v>15</v>
-      </c>
-      <c r="R3" t="n">
+        <v>17</v>
+      </c>
+      <c r="S2" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>